<commit_message>
Clarify LTRP payment as sum of Nominal/6 across plans since 2022.
Document that each year's assigned plan (e.g. 2026 = 70,000) pays Nominal÷6 on Jan 31, and the cash date totals all active 1/6 tranches from LTRP 2022 onward.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/LTRP/LTRP_Sol.xlsx
+++ b/LTRP/LTRP_Sol.xlsx
@@ -64,12 +64,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D6E3F0"/>
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
+        <fgColor rgb="00D6E3F0"/>
       </patternFill>
     </fill>
   </fills>
@@ -99,7 +99,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
@@ -108,9 +108,11 @@
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
@@ -120,12 +122,12 @@
     <xf numFmtId="4" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="4" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="4" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -493,10 +495,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="39" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="1" max="1"/>
     <col width="80" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
@@ -547,110 +549,172 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Duración por plan</t>
+          <t>Fórmula del cobro 31/01</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>6 años (1/6 por año)</t>
+          <t>SUMAR (Valor nominal ÷ 6) de cada plan vigente desde 2022</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Composición del pago</t>
+          <t>Ejemplo plan 2026</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>50% fijo + 50% variable (acción MELI)</t>
+          <t>70.000 ÷ 6 = 11.666,67  +  1/6 de LTRP 2022…2025</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Fecha de pago</t>
+          <t>Duración por plan</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>31/01 del año siguiente al período calculado</t>
+          <t>6 cobros anuales (1/6 por año) en 31/01</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr"/>
-      <c r="B8" s="4" t="inlineStr"/>
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Composición del pago</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>50% fijo + 50% variable (acción MELI)</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>Estimación de pago para 2027</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="n">
-        <v>35332</v>
-      </c>
+      <c r="A9" s="4" t="inlineStr"/>
+      <c r="B9" s="5" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Base total 2027 (factor MELI = 1,0)</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="n">
+          <t>Pago base 31/01/2027 = suma de cinco 1/6</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="n">
         <v>32803.67</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Factor MELI implícito (solo variable)</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="n">
-        <v>1.1542</v>
+          <t xml:space="preserve">  · LTRP 2022 ÷ 6</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="n">
+        <v>5000</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr"/>
-      <c r="B12" s="4" t="inlineStr"/>
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  · LTRP 2023 ÷ 6</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="n">
+        <v>5000</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Total valor nominal planes vigentes</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="n">
-        <v>196822</v>
+          <t xml:space="preserve">  · LTRP 2024 ÷ 6</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="n">
+        <v>5000</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Planes vigentes</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="n">
-        <v>5</v>
+          <t xml:space="preserve">  · LTRP 2025 ÷ 6</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="n">
+        <v>6137</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="inlineStr"/>
-      <c r="B15" s="3" t="inlineStr"/>
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  · LTRP 2026 ÷ 6</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="n">
+        <v>11666.6666666667</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
+          <t>Estimación portal MELI 2027</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>35332</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Factor MELI implícito (solo variable)</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>1.1542</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr"/>
+      <c r="B18" s="6" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>Total valor nominal planes vigentes</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>196822</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Planes vigentes</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr"/>
+      <c r="B21" s="3" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
           <t>Nota</t>
         </is>
       </c>
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>El 50% variable depende de la acción MELI. La estimación del portal puede diferir de la base a factor 1,0. Esta carpeta trackea ingreso por bono; no es gasto CIUDAD/SOL.</t>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>El valor nominal (ej. 70.000) es el plan asignado ese año, NO el cobro anual. El cobro = suma de los ÷6 activos. El 50% variable mueve el total vs la base. Ingreso por bono; no es gasto CIUDAD/SOL.</t>
         </is>
       </c>
     </row>
@@ -729,16 +793,16 @@
       <c r="B2" s="3" t="n">
         <v>2022</v>
       </c>
-      <c r="C2" s="4" t="n">
+      <c r="C2" s="6" t="n">
         <v>30000</v>
       </c>
-      <c r="D2" s="4" t="n">
-        <v>5000</v>
-      </c>
-      <c r="E2" s="4" t="n">
+      <c r="D2" s="6" t="n">
+        <v>5000</v>
+      </c>
+      <c r="E2" s="6" t="n">
         <v>2500</v>
       </c>
-      <c r="F2" s="4" t="n">
+      <c r="F2" s="6" t="n">
         <v>2500</v>
       </c>
       <c r="G2" s="3" t="inlineStr">
@@ -748,7 +812,7 @@
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>Primer pago 31/01/2023 · último 31/01/2028</t>
+          <t>Valor asignado 2022 · aporta 30000/6=5000 en cada 31/01 (2023-2028)</t>
         </is>
       </c>
     </row>
@@ -761,16 +825,16 @@
       <c r="B3" s="3" t="n">
         <v>2023</v>
       </c>
-      <c r="C3" s="4" t="n">
+      <c r="C3" s="6" t="n">
         <v>30000</v>
       </c>
-      <c r="D3" s="4" t="n">
-        <v>5000</v>
-      </c>
-      <c r="E3" s="4" t="n">
+      <c r="D3" s="6" t="n">
+        <v>5000</v>
+      </c>
+      <c r="E3" s="6" t="n">
         <v>2500</v>
       </c>
-      <c r="F3" s="4" t="n">
+      <c r="F3" s="6" t="n">
         <v>2500</v>
       </c>
       <c r="G3" s="3" t="inlineStr">
@@ -780,7 +844,7 @@
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>Primer pago 31/01/2024 · último 31/01/2029</t>
+          <t>Valor asignado 2023 · aporta 30000/6=5000 en cada 31/01 (2024-2029)</t>
         </is>
       </c>
     </row>
@@ -793,16 +857,16 @@
       <c r="B4" s="3" t="n">
         <v>2024</v>
       </c>
-      <c r="C4" s="4" t="n">
+      <c r="C4" s="6" t="n">
         <v>30000</v>
       </c>
-      <c r="D4" s="4" t="n">
-        <v>5000</v>
-      </c>
-      <c r="E4" s="4" t="n">
+      <c r="D4" s="6" t="n">
+        <v>5000</v>
+      </c>
+      <c r="E4" s="6" t="n">
         <v>2500</v>
       </c>
-      <c r="F4" s="4" t="n">
+      <c r="F4" s="6" t="n">
         <v>2500</v>
       </c>
       <c r="G4" s="3" t="inlineStr">
@@ -812,7 +876,7 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>Primer pago 31/01/2025 · último 31/01/2030</t>
+          <t>Valor asignado 2024 · aporta 30000/6=5000 en cada 31/01 (2025-2030)</t>
         </is>
       </c>
     </row>
@@ -825,16 +889,16 @@
       <c r="B5" s="3" t="n">
         <v>2025</v>
       </c>
-      <c r="C5" s="4" t="n">
+      <c r="C5" s="6" t="n">
         <v>36822</v>
       </c>
-      <c r="D5" s="4" t="n">
+      <c r="D5" s="6" t="n">
         <v>6137</v>
       </c>
-      <c r="E5" s="4" t="n">
+      <c r="E5" s="6" t="n">
         <v>3068.5</v>
       </c>
-      <c r="F5" s="4" t="n">
+      <c r="F5" s="6" t="n">
         <v>3068.5</v>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -844,7 +908,7 @@
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>Primer pago 31/01/2026 · último 31/01/2031</t>
+          <t>Valor asignado 2025 · aporta 36822/6=6137 en cada 31/01 (2026-2031)</t>
         </is>
       </c>
     </row>
@@ -857,16 +921,16 @@
       <c r="B6" s="3" t="n">
         <v>2026</v>
       </c>
-      <c r="C6" s="4" t="n">
+      <c r="C6" s="6" t="n">
         <v>70000</v>
       </c>
-      <c r="D6" s="4" t="n">
+      <c r="D6" s="6" t="n">
         <v>11666.6666666667</v>
       </c>
-      <c r="E6" s="4" t="n">
+      <c r="E6" s="6" t="n">
         <v>5833.3333333333</v>
       </c>
-      <c r="F6" s="4" t="n">
+      <c r="F6" s="6" t="n">
         <v>5833.3333333333</v>
       </c>
       <c r="G6" s="3" t="inlineStr">
@@ -876,30 +940,30 @@
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>Primer pago 31/01/2027 · último 31/01/2032</t>
+          <t>Valor asignado 2026 · aporta 70000/6=11666.67 en cada 31/01 (2027-2032) · sumar con 1/6 de 2022..2025</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="inlineStr">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
       <c r="B7" s="3" t="n"/>
-      <c r="C7" s="6">
+      <c r="C7" s="8">
         <f>SUM(C2:C6)</f>
         <v/>
       </c>
-      <c r="D7" s="6">
+      <c r="D7" s="8">
         <f>SUM(D2:D6)</f>
         <v/>
       </c>
-      <c r="E7" s="6">
+      <c r="E7" s="8">
         <f>SUM(E2:E6)</f>
         <v/>
       </c>
-      <c r="F7" s="6">
+      <c r="F7" s="8">
         <f>SUM(F2:F6)</f>
         <v/>
       </c>
@@ -934,262 +998,262 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="7" t="inlineStr">
+      <c r="A1" s="9" t="inlineStr">
         <is>
           <t>Plan</t>
         </is>
       </c>
-      <c r="B1" s="7" t="inlineStr">
+      <c r="B1" s="9" t="inlineStr">
         <is>
           <t>Pago 2023 (31/01/2023)</t>
         </is>
       </c>
-      <c r="C1" s="7" t="inlineStr">
+      <c r="C1" s="9" t="inlineStr">
         <is>
           <t>Pago 2024 (31/01/2024)</t>
         </is>
       </c>
-      <c r="D1" s="7" t="inlineStr">
+      <c r="D1" s="9" t="inlineStr">
         <is>
           <t>Pago 2025 (31/01/2025)</t>
         </is>
       </c>
-      <c r="E1" s="7" t="inlineStr">
+      <c r="E1" s="9" t="inlineStr">
         <is>
           <t>Pago 2026 (31/01/2026)</t>
         </is>
       </c>
-      <c r="F1" s="7" t="inlineStr">
+      <c r="F1" s="9" t="inlineStr">
         <is>
           <t>Pago 2027 (31/01/2027)</t>
         </is>
       </c>
-      <c r="G1" s="7" t="inlineStr">
+      <c r="G1" s="9" t="inlineStr">
         <is>
           <t>Pago 2028 (31/01/2028)</t>
         </is>
       </c>
-      <c r="H1" s="7" t="inlineStr">
+      <c r="H1" s="9" t="inlineStr">
         <is>
           <t>Pago 2029 (31/01/2029)</t>
         </is>
       </c>
-      <c r="I1" s="7" t="inlineStr">
+      <c r="I1" s="9" t="inlineStr">
         <is>
           <t>Pago 2030 (31/01/2030)</t>
         </is>
       </c>
-      <c r="J1" s="7" t="inlineStr">
+      <c r="J1" s="9" t="inlineStr">
         <is>
           <t>Pago 2031 (31/01/2031)</t>
         </is>
       </c>
-      <c r="K1" s="7" t="inlineStr">
+      <c r="K1" s="9" t="inlineStr">
         <is>
           <t>Pago 2032 (31/01/2032)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="8" t="inlineStr">
+      <c r="A2" s="10" t="inlineStr">
         <is>
           <t>LTRP 2022</t>
         </is>
       </c>
-      <c r="B2" s="8" t="inlineStr">
+      <c r="B2" s="10" t="inlineStr">
         <is>
           <t>1/6</t>
         </is>
       </c>
-      <c r="C2" s="8" t="inlineStr">
+      <c r="C2" s="10" t="inlineStr">
         <is>
           <t>2/6</t>
         </is>
       </c>
-      <c r="D2" s="8" t="inlineStr">
+      <c r="D2" s="10" t="inlineStr">
         <is>
           <t>3/6</t>
         </is>
       </c>
-      <c r="E2" s="8" t="inlineStr">
+      <c r="E2" s="10" t="inlineStr">
         <is>
           <t>4/6</t>
         </is>
       </c>
-      <c r="F2" s="8" t="inlineStr">
+      <c r="F2" s="10" t="inlineStr">
         <is>
           <t>5/6</t>
         </is>
       </c>
-      <c r="G2" s="8" t="inlineStr">
+      <c r="G2" s="10" t="inlineStr">
         <is>
           <t>6/6</t>
         </is>
       </c>
-      <c r="H2" s="8" t="inlineStr"/>
-      <c r="I2" s="8" t="inlineStr"/>
-      <c r="J2" s="8" t="inlineStr"/>
-      <c r="K2" s="8" t="inlineStr"/>
+      <c r="H2" s="10" t="inlineStr"/>
+      <c r="I2" s="10" t="inlineStr"/>
+      <c r="J2" s="10" t="inlineStr"/>
+      <c r="K2" s="10" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="inlineStr">
+      <c r="A3" s="10" t="inlineStr">
         <is>
           <t>LTRP 2023</t>
         </is>
       </c>
-      <c r="B3" s="8" t="inlineStr"/>
-      <c r="C3" s="8" t="inlineStr">
+      <c r="B3" s="10" t="inlineStr"/>
+      <c r="C3" s="10" t="inlineStr">
         <is>
           <t>1/6</t>
         </is>
       </c>
-      <c r="D3" s="8" t="inlineStr">
+      <c r="D3" s="10" t="inlineStr">
         <is>
           <t>2/6</t>
         </is>
       </c>
-      <c r="E3" s="8" t="inlineStr">
+      <c r="E3" s="10" t="inlineStr">
         <is>
           <t>3/6</t>
         </is>
       </c>
-      <c r="F3" s="8" t="inlineStr">
+      <c r="F3" s="10" t="inlineStr">
         <is>
           <t>4/6</t>
         </is>
       </c>
-      <c r="G3" s="8" t="inlineStr">
+      <c r="G3" s="10" t="inlineStr">
         <is>
           <t>5/6</t>
         </is>
       </c>
-      <c r="H3" s="8" t="inlineStr">
+      <c r="H3" s="10" t="inlineStr">
         <is>
           <t>6/6</t>
         </is>
       </c>
-      <c r="I3" s="8" t="inlineStr"/>
-      <c r="J3" s="8" t="inlineStr"/>
-      <c r="K3" s="8" t="inlineStr"/>
+      <c r="I3" s="10" t="inlineStr"/>
+      <c r="J3" s="10" t="inlineStr"/>
+      <c r="K3" s="10" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="inlineStr">
+      <c r="A4" s="10" t="inlineStr">
         <is>
           <t>LTRP 2024</t>
         </is>
       </c>
-      <c r="B4" s="8" t="inlineStr"/>
-      <c r="C4" s="8" t="inlineStr"/>
-      <c r="D4" s="8" t="inlineStr">
+      <c r="B4" s="10" t="inlineStr"/>
+      <c r="C4" s="10" t="inlineStr"/>
+      <c r="D4" s="10" t="inlineStr">
         <is>
           <t>1/6</t>
         </is>
       </c>
-      <c r="E4" s="8" t="inlineStr">
+      <c r="E4" s="10" t="inlineStr">
         <is>
           <t>2/6</t>
         </is>
       </c>
-      <c r="F4" s="8" t="inlineStr">
+      <c r="F4" s="10" t="inlineStr">
         <is>
           <t>3/6</t>
         </is>
       </c>
-      <c r="G4" s="8" t="inlineStr">
+      <c r="G4" s="10" t="inlineStr">
         <is>
           <t>4/6</t>
         </is>
       </c>
-      <c r="H4" s="8" t="inlineStr">
+      <c r="H4" s="10" t="inlineStr">
         <is>
           <t>5/6</t>
         </is>
       </c>
-      <c r="I4" s="8" t="inlineStr">
+      <c r="I4" s="10" t="inlineStr">
         <is>
           <t>6/6</t>
         </is>
       </c>
-      <c r="J4" s="8" t="inlineStr"/>
-      <c r="K4" s="8" t="inlineStr"/>
+      <c r="J4" s="10" t="inlineStr"/>
+      <c r="K4" s="10" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="A5" s="10" t="inlineStr">
         <is>
           <t>LTRP 2025</t>
         </is>
       </c>
-      <c r="B5" s="8" t="inlineStr"/>
-      <c r="C5" s="8" t="inlineStr"/>
-      <c r="D5" s="8" t="inlineStr"/>
-      <c r="E5" s="8" t="inlineStr">
+      <c r="B5" s="10" t="inlineStr"/>
+      <c r="C5" s="10" t="inlineStr"/>
+      <c r="D5" s="10" t="inlineStr"/>
+      <c r="E5" s="10" t="inlineStr">
         <is>
           <t>1/6</t>
         </is>
       </c>
-      <c r="F5" s="8" t="inlineStr">
+      <c r="F5" s="10" t="inlineStr">
         <is>
           <t>2/6</t>
         </is>
       </c>
-      <c r="G5" s="8" t="inlineStr">
+      <c r="G5" s="10" t="inlineStr">
         <is>
           <t>3/6</t>
         </is>
       </c>
-      <c r="H5" s="8" t="inlineStr">
+      <c r="H5" s="10" t="inlineStr">
         <is>
           <t>4/6</t>
         </is>
       </c>
-      <c r="I5" s="8" t="inlineStr">
+      <c r="I5" s="10" t="inlineStr">
         <is>
           <t>5/6</t>
         </is>
       </c>
-      <c r="J5" s="8" t="inlineStr">
+      <c r="J5" s="10" t="inlineStr">
         <is>
           <t>6/6</t>
         </is>
       </c>
-      <c r="K5" s="8" t="inlineStr"/>
+      <c r="K5" s="10" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="inlineStr">
+      <c r="A6" s="10" t="inlineStr">
         <is>
           <t>LTRP 2026</t>
         </is>
       </c>
-      <c r="B6" s="8" t="inlineStr"/>
-      <c r="C6" s="8" t="inlineStr"/>
-      <c r="D6" s="8" t="inlineStr"/>
-      <c r="E6" s="8" t="inlineStr"/>
-      <c r="F6" s="8" t="inlineStr">
+      <c r="B6" s="10" t="inlineStr"/>
+      <c r="C6" s="10" t="inlineStr"/>
+      <c r="D6" s="10" t="inlineStr"/>
+      <c r="E6" s="10" t="inlineStr"/>
+      <c r="F6" s="10" t="inlineStr">
         <is>
           <t>1/6</t>
         </is>
       </c>
-      <c r="G6" s="8" t="inlineStr">
+      <c r="G6" s="10" t="inlineStr">
         <is>
           <t>2/6</t>
         </is>
       </c>
-      <c r="H6" s="8" t="inlineStr">
+      <c r="H6" s="10" t="inlineStr">
         <is>
           <t>3/6</t>
         </is>
       </c>
-      <c r="I6" s="8" t="inlineStr">
+      <c r="I6" s="10" t="inlineStr">
         <is>
           <t>4/6</t>
         </is>
       </c>
-      <c r="J6" s="8" t="inlineStr">
+      <c r="J6" s="10" t="inlineStr">
         <is>
           <t>5/6</t>
         </is>
       </c>
-      <c r="K6" s="8" t="inlineStr">
+      <c r="K6" s="10" t="inlineStr">
         <is>
           <t>6/6</t>
         </is>
@@ -1297,32 +1361,32 @@
           <t>LTRP 2022</t>
         </is>
       </c>
-      <c r="B2" s="9" t="n">
+      <c r="B2" s="11" t="n">
         <v>30000</v>
       </c>
-      <c r="C2" s="9" t="n">
-        <v>5000</v>
-      </c>
-      <c r="D2" s="9" t="n">
-        <v>5000</v>
-      </c>
-      <c r="E2" s="9" t="n">
-        <v>5000</v>
-      </c>
-      <c r="F2" s="9" t="n">
-        <v>5000</v>
-      </c>
-      <c r="G2" s="9" t="n">
-        <v>5000</v>
-      </c>
-      <c r="H2" s="9" t="n">
-        <v>5000</v>
-      </c>
-      <c r="I2" s="8" t="n"/>
-      <c r="J2" s="8" t="n"/>
-      <c r="K2" s="8" t="n"/>
-      <c r="L2" s="8" t="n"/>
-      <c r="M2" s="9" t="n">
+      <c r="C2" s="11" t="n">
+        <v>5000</v>
+      </c>
+      <c r="D2" s="11" t="n">
+        <v>5000</v>
+      </c>
+      <c r="E2" s="11" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F2" s="11" t="n">
+        <v>5000</v>
+      </c>
+      <c r="G2" s="11" t="n">
+        <v>5000</v>
+      </c>
+      <c r="H2" s="11" t="n">
+        <v>5000</v>
+      </c>
+      <c r="I2" s="10" t="n"/>
+      <c r="J2" s="10" t="n"/>
+      <c r="K2" s="10" t="n"/>
+      <c r="L2" s="10" t="n"/>
+      <c r="M2" s="11" t="n">
         <v>30000</v>
       </c>
     </row>
@@ -1332,32 +1396,32 @@
           <t>LTRP 2023</t>
         </is>
       </c>
-      <c r="B3" s="9" t="n">
+      <c r="B3" s="11" t="n">
         <v>30000</v>
       </c>
-      <c r="C3" s="8" t="n"/>
-      <c r="D3" s="9" t="n">
-        <v>5000</v>
-      </c>
-      <c r="E3" s="9" t="n">
-        <v>5000</v>
-      </c>
-      <c r="F3" s="9" t="n">
-        <v>5000</v>
-      </c>
-      <c r="G3" s="9" t="n">
-        <v>5000</v>
-      </c>
-      <c r="H3" s="9" t="n">
-        <v>5000</v>
-      </c>
-      <c r="I3" s="9" t="n">
-        <v>5000</v>
-      </c>
-      <c r="J3" s="8" t="n"/>
-      <c r="K3" s="8" t="n"/>
-      <c r="L3" s="8" t="n"/>
-      <c r="M3" s="9" t="n">
+      <c r="C3" s="10" t="n"/>
+      <c r="D3" s="11" t="n">
+        <v>5000</v>
+      </c>
+      <c r="E3" s="11" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F3" s="11" t="n">
+        <v>5000</v>
+      </c>
+      <c r="G3" s="11" t="n">
+        <v>5000</v>
+      </c>
+      <c r="H3" s="11" t="n">
+        <v>5000</v>
+      </c>
+      <c r="I3" s="11" t="n">
+        <v>5000</v>
+      </c>
+      <c r="J3" s="10" t="n"/>
+      <c r="K3" s="10" t="n"/>
+      <c r="L3" s="10" t="n"/>
+      <c r="M3" s="11" t="n">
         <v>30000</v>
       </c>
     </row>
@@ -1367,32 +1431,32 @@
           <t>LTRP 2024</t>
         </is>
       </c>
-      <c r="B4" s="9" t="n">
+      <c r="B4" s="11" t="n">
         <v>30000</v>
       </c>
-      <c r="C4" s="8" t="n"/>
-      <c r="D4" s="8" t="n"/>
-      <c r="E4" s="9" t="n">
-        <v>5000</v>
-      </c>
-      <c r="F4" s="9" t="n">
-        <v>5000</v>
-      </c>
-      <c r="G4" s="9" t="n">
-        <v>5000</v>
-      </c>
-      <c r="H4" s="9" t="n">
-        <v>5000</v>
-      </c>
-      <c r="I4" s="9" t="n">
-        <v>5000</v>
-      </c>
-      <c r="J4" s="9" t="n">
-        <v>5000</v>
-      </c>
-      <c r="K4" s="8" t="n"/>
-      <c r="L4" s="8" t="n"/>
-      <c r="M4" s="9" t="n">
+      <c r="C4" s="10" t="n"/>
+      <c r="D4" s="10" t="n"/>
+      <c r="E4" s="11" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F4" s="11" t="n">
+        <v>5000</v>
+      </c>
+      <c r="G4" s="11" t="n">
+        <v>5000</v>
+      </c>
+      <c r="H4" s="11" t="n">
+        <v>5000</v>
+      </c>
+      <c r="I4" s="11" t="n">
+        <v>5000</v>
+      </c>
+      <c r="J4" s="11" t="n">
+        <v>5000</v>
+      </c>
+      <c r="K4" s="10" t="n"/>
+      <c r="L4" s="10" t="n"/>
+      <c r="M4" s="11" t="n">
         <v>30000</v>
       </c>
     </row>
@@ -1402,32 +1466,32 @@
           <t>LTRP 2025</t>
         </is>
       </c>
-      <c r="B5" s="9" t="n">
+      <c r="B5" s="11" t="n">
         <v>36822</v>
       </c>
-      <c r="C5" s="8" t="n"/>
-      <c r="D5" s="8" t="n"/>
-      <c r="E5" s="8" t="n"/>
-      <c r="F5" s="9" t="n">
+      <c r="C5" s="10" t="n"/>
+      <c r="D5" s="10" t="n"/>
+      <c r="E5" s="10" t="n"/>
+      <c r="F5" s="11" t="n">
         <v>6137</v>
       </c>
-      <c r="G5" s="9" t="n">
+      <c r="G5" s="11" t="n">
         <v>6137</v>
       </c>
-      <c r="H5" s="9" t="n">
+      <c r="H5" s="11" t="n">
         <v>6137</v>
       </c>
-      <c r="I5" s="9" t="n">
+      <c r="I5" s="11" t="n">
         <v>6137</v>
       </c>
-      <c r="J5" s="9" t="n">
+      <c r="J5" s="11" t="n">
         <v>6137</v>
       </c>
-      <c r="K5" s="9" t="n">
+      <c r="K5" s="11" t="n">
         <v>6137</v>
       </c>
-      <c r="L5" s="8" t="n"/>
-      <c r="M5" s="9" t="n">
+      <c r="L5" s="10" t="n"/>
+      <c r="M5" s="11" t="n">
         <v>36822</v>
       </c>
     </row>
@@ -1437,76 +1501,76 @@
           <t>LTRP 2026</t>
         </is>
       </c>
-      <c r="B6" s="9" t="n">
+      <c r="B6" s="11" t="n">
         <v>70000</v>
       </c>
-      <c r="C6" s="8" t="n"/>
-      <c r="D6" s="8" t="n"/>
-      <c r="E6" s="8" t="n"/>
-      <c r="F6" s="8" t="n"/>
-      <c r="G6" s="9" t="n">
+      <c r="C6" s="10" t="n"/>
+      <c r="D6" s="10" t="n"/>
+      <c r="E6" s="10" t="n"/>
+      <c r="F6" s="10" t="n"/>
+      <c r="G6" s="11" t="n">
         <v>11666.66666666667</v>
       </c>
-      <c r="H6" s="9" t="n">
+      <c r="H6" s="11" t="n">
         <v>11666.66666666667</v>
       </c>
-      <c r="I6" s="9" t="n">
+      <c r="I6" s="11" t="n">
         <v>11666.66666666667</v>
       </c>
-      <c r="J6" s="9" t="n">
+      <c r="J6" s="11" t="n">
         <v>11666.66666666667</v>
       </c>
-      <c r="K6" s="9" t="n">
+      <c r="K6" s="11" t="n">
         <v>11666.66666666667</v>
       </c>
-      <c r="L6" s="9" t="n">
+      <c r="L6" s="11" t="n">
         <v>11666.66666666667</v>
       </c>
-      <c r="M6" s="9" t="n">
+      <c r="M6" s="11" t="n">
         <v>70000</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="inlineStr">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B7" s="10">
+      <c r="B7" s="12">
         <f>SUM(B2:B6)</f>
         <v/>
       </c>
-      <c r="C7" s="10" t="n">
-        <v>5000</v>
-      </c>
-      <c r="D7" s="10" t="n">
+      <c r="C7" s="12" t="n">
+        <v>5000</v>
+      </c>
+      <c r="D7" s="12" t="n">
         <v>10000</v>
       </c>
-      <c r="E7" s="10" t="n">
+      <c r="E7" s="12" t="n">
         <v>15000</v>
       </c>
-      <c r="F7" s="10" t="n">
+      <c r="F7" s="12" t="n">
         <v>21137</v>
       </c>
-      <c r="G7" s="10" t="n">
+      <c r="G7" s="12" t="n">
         <v>32803.66666666666</v>
       </c>
-      <c r="H7" s="10" t="n">
+      <c r="H7" s="12" t="n">
         <v>32803.66666666666</v>
       </c>
-      <c r="I7" s="10" t="n">
+      <c r="I7" s="12" t="n">
         <v>27803.66666666666</v>
       </c>
-      <c r="J7" s="10" t="n">
+      <c r="J7" s="12" t="n">
         <v>22803.66666666666</v>
       </c>
-      <c r="K7" s="10" t="n">
+      <c r="K7" s="12" t="n">
         <v>17803.66666666666</v>
       </c>
-      <c r="L7" s="10" t="n">
+      <c r="L7" s="12" t="n">
         <v>11666.66666666667</v>
       </c>
-      <c r="M7" s="10" t="n">
+      <c r="M7" s="12" t="n">
         <v>196822</v>
       </c>
     </row>
@@ -1533,7 +1597,7 @@
     <col width="21" customWidth="1" min="7" max="7"/>
     <col width="34" customWidth="1" min="8" max="8"/>
     <col width="22" customWidth="1" min="9" max="9"/>
-    <col width="52" customWidth="1" min="10" max="10"/>
+    <col width="55" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1600,13 +1664,13 @@
       <c r="C2" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="D2" s="4" t="n">
+      <c r="D2" s="6" t="n">
         <v>2500</v>
       </c>
-      <c r="E2" s="4" t="n">
+      <c r="E2" s="6" t="n">
         <v>2500</v>
       </c>
-      <c r="F2" s="4" t="n">
+      <c r="F2" s="6" t="n">
         <v>5000</v>
       </c>
       <c r="G2" s="3" t="n"/>
@@ -1630,13 +1694,13 @@
       <c r="C3" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="D3" s="4" t="n">
-        <v>5000</v>
-      </c>
-      <c r="E3" s="4" t="n">
-        <v>5000</v>
-      </c>
-      <c r="F3" s="4" t="n">
+      <c r="D3" s="6" t="n">
+        <v>5000</v>
+      </c>
+      <c r="E3" s="6" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F3" s="6" t="n">
         <v>10000</v>
       </c>
       <c r="G3" s="3" t="n"/>
@@ -1660,13 +1724,13 @@
       <c r="C4" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="D4" s="4" t="n">
+      <c r="D4" s="6" t="n">
         <v>7500</v>
       </c>
-      <c r="E4" s="4" t="n">
+      <c r="E4" s="6" t="n">
         <v>7500</v>
       </c>
-      <c r="F4" s="4" t="n">
+      <c r="F4" s="6" t="n">
         <v>15000</v>
       </c>
       <c r="G4" s="3" t="n"/>
@@ -1690,13 +1754,13 @@
       <c r="C5" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="D5" s="4" t="n">
+      <c r="D5" s="6" t="n">
         <v>10568.5</v>
       </c>
-      <c r="E5" s="4" t="n">
+      <c r="E5" s="6" t="n">
         <v>10568.5</v>
       </c>
-      <c r="F5" s="4" t="n">
+      <c r="F5" s="6" t="n">
         <v>21137</v>
       </c>
       <c r="G5" s="3" t="n"/>
@@ -1709,40 +1773,40 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="11" t="n">
+      <c r="A6" s="13" t="n">
         <v>2027</v>
       </c>
-      <c r="B6" s="11" t="inlineStr">
+      <c r="B6" s="13" t="inlineStr">
         <is>
           <t>2027-01-31</t>
         </is>
       </c>
-      <c r="C6" s="11" t="n">
+      <c r="C6" s="13" t="n">
         <v>5</v>
       </c>
-      <c r="D6" s="12" t="n">
+      <c r="D6" s="14" t="n">
         <v>16401.83</v>
       </c>
-      <c r="E6" s="12" t="n">
+      <c r="E6" s="14" t="n">
         <v>16401.83</v>
       </c>
-      <c r="F6" s="12" t="n">
+      <c r="F6" s="14" t="n">
         <v>32803.67</v>
       </c>
-      <c r="G6" s="12" t="n">
+      <c r="G6" s="14" t="n">
         <v>35332</v>
       </c>
-      <c r="H6" s="13" t="n">
+      <c r="H6" s="15" t="n">
         <v>1.1542</v>
       </c>
-      <c r="I6" s="11" t="inlineStr">
+      <c r="I6" s="13" t="inlineStr">
         <is>
           <t>2026-08</t>
         </is>
       </c>
-      <c r="J6" s="11" t="inlineStr">
-        <is>
-          <t>Estimación portal MELI agosto 2026 · USD 35.332</t>
+      <c r="J6" s="13" t="inlineStr">
+        <is>
+          <t>Suma 1/6 de LTRP 2022..2026 = 5000+5000+5000+6137+11666.67 · portal 35.332</t>
         </is>
       </c>
     </row>
@@ -1758,13 +1822,13 @@
       <c r="C7" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="D7" s="4" t="n">
+      <c r="D7" s="6" t="n">
         <v>16401.83</v>
       </c>
-      <c r="E7" s="4" t="n">
+      <c r="E7" s="6" t="n">
         <v>16401.83</v>
       </c>
-      <c r="F7" s="4" t="n">
+      <c r="F7" s="6" t="n">
         <v>32803.67</v>
       </c>
       <c r="G7" s="3" t="n"/>
@@ -1788,13 +1852,13 @@
       <c r="C8" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="D8" s="4" t="n">
+      <c r="D8" s="6" t="n">
         <v>13901.83</v>
       </c>
-      <c r="E8" s="4" t="n">
+      <c r="E8" s="6" t="n">
         <v>13901.83</v>
       </c>
-      <c r="F8" s="4" t="n">
+      <c r="F8" s="6" t="n">
         <v>27803.67</v>
       </c>
       <c r="G8" s="3" t="n"/>
@@ -1818,13 +1882,13 @@
       <c r="C9" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="D9" s="4" t="n">
+      <c r="D9" s="6" t="n">
         <v>11401.83</v>
       </c>
-      <c r="E9" s="4" t="n">
+      <c r="E9" s="6" t="n">
         <v>11401.83</v>
       </c>
-      <c r="F9" s="4" t="n">
+      <c r="F9" s="6" t="n">
         <v>22803.67</v>
       </c>
       <c r="G9" s="3" t="n"/>
@@ -1848,13 +1912,13 @@
       <c r="C10" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="D10" s="4" t="n">
+      <c r="D10" s="6" t="n">
         <v>8901.83</v>
       </c>
-      <c r="E10" s="4" t="n">
+      <c r="E10" s="6" t="n">
         <v>8901.83</v>
       </c>
-      <c r="F10" s="4" t="n">
+      <c r="F10" s="6" t="n">
         <v>17803.67</v>
       </c>
       <c r="G10" s="3" t="n"/>
@@ -1878,13 +1942,13 @@
       <c r="C11" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="D11" s="4" t="n">
+      <c r="D11" s="6" t="n">
         <v>5833.33</v>
       </c>
-      <c r="E11" s="4" t="n">
+      <c r="E11" s="6" t="n">
         <v>5833.33</v>
       </c>
-      <c r="F11" s="4" t="n">
+      <c r="F11" s="6" t="n">
         <v>11666.67</v>
       </c>
       <c r="G11" s="3" t="n"/>
@@ -1907,11 +1971,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="44" customWidth="1" min="1" max="1"/>
-    <col width="70" customWidth="1" min="2" max="2"/>
+    <col width="65" customWidth="1" min="1" max="1"/>
+    <col width="66" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="19" customWidth="1" min="4" max="4"/>
     <col width="23" customWidth="1" min="5" max="5"/>
@@ -1920,9 +1984,9 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="14" t="inlineStr">
-        <is>
-          <t>Detalle estimación pago 31/01/2027</t>
+      <c r="A1" s="16" t="inlineStr">
+        <is>
+          <t>Pago 31/01/2027 = suma de (Nominal ÷ 6) de cada plan desde 2022</t>
         </is>
       </c>
     </row>
@@ -1935,12 +1999,12 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Año vesting</t>
+          <t>Valor nominal USD</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Tramo 1/6 USD</t>
+          <t>Nominal ÷ 6</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -1970,24 +2034,22 @@
           <t>LTRP 2022</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>5/6</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="n">
-        <v>5000</v>
-      </c>
-      <c r="D4" s="4" t="n">
+      <c r="B4" s="6" t="n">
+        <v>30000</v>
+      </c>
+      <c r="C4" s="6" t="n">
+        <v>5000</v>
+      </c>
+      <c r="D4" s="6" t="n">
         <v>2500</v>
       </c>
-      <c r="E4" s="4" t="n">
+      <c r="E4" s="6" t="n">
         <v>2500</v>
       </c>
-      <c r="F4" s="4" t="n">
+      <c r="F4" s="6" t="n">
         <v>2885.5</v>
       </c>
-      <c r="G4" s="4" t="n">
+      <c r="G4" s="6" t="n">
         <v>5385.5</v>
       </c>
     </row>
@@ -1997,24 +2059,22 @@
           <t>LTRP 2023</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>4/6</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="n">
-        <v>5000</v>
-      </c>
-      <c r="D5" s="4" t="n">
+      <c r="B5" s="6" t="n">
+        <v>30000</v>
+      </c>
+      <c r="C5" s="6" t="n">
+        <v>5000</v>
+      </c>
+      <c r="D5" s="6" t="n">
         <v>2500</v>
       </c>
-      <c r="E5" s="4" t="n">
+      <c r="E5" s="6" t="n">
         <v>2500</v>
       </c>
-      <c r="F5" s="4" t="n">
+      <c r="F5" s="6" t="n">
         <v>2885.5</v>
       </c>
-      <c r="G5" s="4" t="n">
+      <c r="G5" s="6" t="n">
         <v>5385.5</v>
       </c>
     </row>
@@ -2024,24 +2084,22 @@
           <t>LTRP 2024</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>3/6</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="n">
-        <v>5000</v>
-      </c>
-      <c r="D6" s="4" t="n">
+      <c r="B6" s="6" t="n">
+        <v>30000</v>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>5000</v>
+      </c>
+      <c r="D6" s="6" t="n">
         <v>2500</v>
       </c>
-      <c r="E6" s="4" t="n">
+      <c r="E6" s="6" t="n">
         <v>2500</v>
       </c>
-      <c r="F6" s="4" t="n">
+      <c r="F6" s="6" t="n">
         <v>2885.5</v>
       </c>
-      <c r="G6" s="4" t="n">
+      <c r="G6" s="6" t="n">
         <v>5385.5</v>
       </c>
     </row>
@@ -2051,24 +2109,22 @@
           <t>LTRP 2025</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>2/6</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="n">
+      <c r="B7" s="6" t="n">
+        <v>36822</v>
+      </c>
+      <c r="C7" s="6" t="n">
         <v>6137</v>
       </c>
-      <c r="D7" s="4" t="n">
+      <c r="D7" s="6" t="n">
         <v>3068.5</v>
       </c>
-      <c r="E7" s="4" t="n">
+      <c r="E7" s="6" t="n">
         <v>3068.5</v>
       </c>
-      <c r="F7" s="4" t="n">
+      <c r="F7" s="6" t="n">
         <v>3541.6627</v>
       </c>
-      <c r="G7" s="4" t="n">
+      <c r="G7" s="6" t="n">
         <v>6610.1627</v>
       </c>
     </row>
@@ -2078,51 +2134,52 @@
           <t>LTRP 2026</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>1/6</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="n">
+      <c r="B8" s="6" t="n">
+        <v>70000</v>
+      </c>
+      <c r="C8" s="6" t="n">
         <v>11666.66666666667</v>
       </c>
-      <c r="D8" s="4" t="n">
+      <c r="D8" s="6" t="n">
         <v>5833.333333333333</v>
       </c>
-      <c r="E8" s="4" t="n">
+      <c r="E8" s="6" t="n">
         <v>5833.333333333333</v>
       </c>
-      <c r="F8" s="4" t="n">
+      <c r="F8" s="6" t="n">
         <v>6732.833333333332</v>
       </c>
-      <c r="G8" s="4" t="n">
+      <c r="G8" s="6" t="n">
         <v>12566.16666666666</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr"/>
-      <c r="C9" s="6">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>SUMA (pago base 31/01/2027)</t>
+        </is>
+      </c>
+      <c r="B9" s="8">
+        <f>SUM(B4:B8)</f>
+        <v/>
+      </c>
+      <c r="C9" s="8">
         <f>SUM(C4:C8)</f>
         <v/>
       </c>
-      <c r="D9" s="6">
+      <c r="D9" s="8">
         <f>SUM(D4:D8)</f>
         <v/>
       </c>
-      <c r="E9" s="6">
+      <c r="E9" s="8">
         <f>SUM(E4:E8)</f>
         <v/>
       </c>
-      <c r="F9" s="6">
+      <c r="F9" s="8">
         <f>SUM(F4:F8)</f>
         <v/>
       </c>
-      <c r="G9" s="6">
+      <c r="G9" s="8">
         <f>SUM(G4:G8)</f>
         <v/>
       </c>
@@ -2131,44 +2188,63 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Estimación portal MELI (agosto 2026)</t>
-        </is>
-      </c>
-      <c r="B11" s="15" t="n">
-        <v>35332</v>
+          <t>Fórmula</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Pago base = 30000/6 + 30000/6 + 30000/6 + 36822/6 + 70000/6</t>
+        </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Factor MELI usado en esta hoja (implícito)</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>1.1542</v>
+      <c r="A12" t="inlineStr"/>
+      <c r="B12">
+        <f> 5.000 + 5.000 + 5.000 + 6.137 + 11.666,67 = 32.803,67</f>
+        <v/>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>*Variable estimado</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Variable base × factor MELI implícito derivado de 35.332 vs base 32.803,67</t>
-        </is>
+          <t>Estimación portal MELI (agosto 2026)</t>
+        </is>
+      </c>
+      <c r="B13" s="17" t="n">
+        <v>35332</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Fórmula</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Pago = (Nominal/6)×50% + (Nominal/6)×50%×factor_MELI</t>
+          <t>Factor MELI usado en esta hoja (implícito)</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>1.1542</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>*Variable estimado</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Variable base × factor MELI implícito (35.332 vs base 32.803,67)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Pago final</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>(suma ÷6)×50% fijo + (suma ÷6)×50%×factor_MELI</t>
         </is>
       </c>
     </row>

</xml_diff>